<commit_message>
ajustes no cadastro para salvar corretamente campos qtde de alunos e se possui espaco para horta
</commit_message>
<xml_diff>
--- a/escolas.xlsx
+++ b/escolas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alunouninter-my.sharepoint.com/personal/3554672_alunouninter_com/Documents/CIENCIA DE DADOS/MATERIAS FASE A  II/ATIVIDADE EXTENSIONISTA TECNOLOGIA APLICADA A INCLUSAO DIGITAL II/PROJETO FINAL/raizes-do-amanha1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51B82E22-B149-4E5A-B855-CB6278437E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{51B82E22-B149-4E5A-B855-CB6278437E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A076CB3-F791-4D75-BE86-EE1893A98948}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8E12FB3C-BA5E-4EBE-926F-D9D608AA2FD2}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>NOME DA ESCOLA</t>
   </si>
@@ -64,9 +64,6 @@
     <t>(51) 3341-3210</t>
   </si>
   <si>
-    <t>51 a 200</t>
-  </si>
-  <si>
     <t>Núcleo EJA e CP Darcy Ribeiro</t>
   </si>
   <si>
@@ -101,6 +98,15 @@
   </si>
   <si>
     <t>domdiogodesouza01cre@educar.rs.gov.br</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESPONSAVEL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIPO </t>
+  </si>
+  <si>
+    <t>ESCOLA</t>
   </si>
 </sst>
 </file>
@@ -961,123 +967,153 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{221C232B-1031-41BB-8E63-06324F66B872}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="38.109375" customWidth="1"/>
+    <col min="4" max="4" width="30.88671875" customWidth="1"/>
+    <col min="5" max="5" width="35.88671875" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="42.5546875" customWidth="1"/>
+    <col min="8" max="8" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>317</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3">
+        <v>200</v>
+      </c>
+      <c r="H3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4">
+        <v>370</v>
+      </c>
+      <c r="H4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="F4" t="s">
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5">
+        <v>331</v>
+      </c>
+      <c r="H5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="E5">
-        <v>331</v>
-      </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>24</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6">
+      <c r="G6">
         <v>866</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>